<commit_message>
All 8 articles for the goodjournalism and also the old 20202 articles with new gradings
</commit_message>
<xml_diff>
--- a/GoodJournalism/Op-Ed_Articles.xlsx
+++ b/GoodJournalism/Op-Ed_Articles.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ML\LLMS\GoodJournalism\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D87FDB17-B150-41A4-A5DF-694819492467}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C09770F3-3C6B-4F5C-8D14-C5F1760A7EBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>Article Link</t>
   </si>
@@ -90,16 +90,132 @@
 The globalization of finance and corporate ownership, and the increasing mobility of capital necessarily involved, can produce huge gains in wealth and promote peace by tying interests together across borders. But it has also entangled investors, banks, and corporations in liberal democracies with oligarchs and foreign bagmen acting in the corrupt, illiberal interests of authoritarian despots. Indeed, the president of the United States may well be a compromised agent of authoritarian kleptocrats. We should see the risk of incentivizing America’s mega-rich to even hide more of their assets in the global shadow economy in the light of this truly terrifying fact.
 You don’t need to agree with Elizabeth Warren about taxes to see her, as I do, as the greatest enemy of corruption, graft, and capitalist self-dealing in the U.S. Senate, and its most compelling advocate of clean government and democratic reform. But a wealth tax intended to shore up democracy risks doing the reverse by turbo-charging the shadow economy and aligning the interests of the non-crooked American super-rich with the interests of the despots, gangsters, and native grifters who have already shaken the foundation of our democracy from the backchannels of global dark money.  </t>
   </si>
+  <si>
+    <t>https://www.nytimes.com/2025/10/31/opinion/shutdown-snap-trump-deal.html</t>
+  </si>
+  <si>
+    <t>President Trump has played fast and loose with federal law during the current government shutdown to fund the things he considers important. He has found ways to pay military service members and F.B.I. agents. He has distributed tariff revenues to women with small children and arranged billions of dollars in financial support for Argentina. He has even ordered the Interior Department to keep federal lands open for hunting.
+And what has Mr. Trump refused to fund?
+As the shutdown enters its second month, the president still will not agree to an extension of the federal tax credits that allow millions of Americans to afford health insurance. Last week the Trump administration also said it would stop distributing food stamps to more than 40 million lower-income families, declining to tap the program’s emergency reserve fund.
+A federal judge in Rhode Island intervened on Friday, ordering the administration to use the program’s reserves. A second federal judge, in Massachusetts, indicated that she was also prepared to rule against the administration if it did not agree to continue distributing food stamps. We urge the administration to abide by the decision and allow millions of Americans to receive food aid.
+The government has never paused the distribution of food stamps, even during past shutdowns, and the threat is just one of the ways this shutdown is causing pain. More than a million federal workers are not being paid. The Small Business Administration is not making loans. Regulators are not conducting many routine safety inspections of food processing plants.
+Mr. Trump and his congressional allies could end all of this by doing what they should have done months ago: making a deal. Under current Senate rules, Republicans manifestly do not have enough votes to pass a funding bill on their own, and it is absurd that they continue to insist that Democrats should simply acquiesce. The hard work of governing in a democracy is hammering out a compromise.
+Mr. Trump already has sought to pile pressure on Democrats by suspending funding for projects in blue states, including the important Hudson River train tunnel between New Jersey and New York and mass transit in Chicago. The attempt to raise the stakes by suspending the distribution of food stamps is unconscionable. The administration would literally be keeping food from the mouths of hungry children. Food stamps, formally known as the Supplemental Nutrition Assistance Program, provide a monthly credit to millions of households that do not make enough money to feed themselves. Many recipients work low-wage jobs. Others are disabled or elderly.
+The Agriculture Department, which administers the program, has an emergency reserve of $5.5 billion that could have been used to maintain benefits. During the last long shutdown, in Mr. Trump’s first term, the department said it would tap that fund to delay any interruption in the distribution of benefits. As recently as Sept. 30, the day before the current shutdown began, the department said that remained its plan. Instead, however, the Trump administration insisted the reserve was “not legally available” because it was meant for the aftermath of natural disasters.
+Democrats, for their part, have remained united in their insistence that Republicans must agree to extend the Affordable Care Act tax credits as part of any funding bill. They have resisted despite the pain Mr. Trump is causing because the credits are worth fighting for. The cost of health insurance plans sold through the A.C.A. marketplaces is set to rise sharply next year. The expiring tax credits would have shielded buyers from most of the increase. Without the credits, the average amount that people must pay each month is expected to rise to $159 from $74, according to KFF, a health research group.
+For many, the difference — about $1,000 a year on average — would make the plans unaffordable. Indeed, one reason the premiums are rising is that insurers anticipate the cost increases will cause a significant number of relatively healthy people to drop their insurance, raising costs for everyone else.
+Republicans say their party has become the party of the American working class. But many working families rely on the tax credits to afford health insurance. And many of those same families rely on food stamps to put enough food on the table. Mr. Trump can serve their needs by demonstrating his skills as a negotiator. It’s time to make a deal.</t>
+  </si>
+  <si>
+    <t>https://www.nytimes.com/2025/10/27/opinion/immigration-enforcement-latino-discrimination.html</t>
+  </si>
+  <si>
+    <t>The Trump administration’s crackdown on illegal immigration has become a campaign of discrimination against Latinos. Federal agents are rounding up people with brown skin, catching both U.S. citizens and legal immigrants in their dragnet. Some Latinos are now afraid to speak Spanish or listen to Spanish music in public. Some are missing Mass and staying home on Sundays, or asking friends to pick up their children from school. American citizens are living in fear of a government that is sworn to protect their liberties and keep them safe.
+They have reason to fear. In President Trump’s anti-immigration blitz, federal agents have repeatedly violated civil liberties and humiliated people. Masked officials have shattered car windows and pulled out drivers, leaving children sobbing in back seats. In the middle of the night in Chicago, agents with rifles swarmed an apartment building, broke down doors and dragged people from their homes in handcuffs. Dozens of those taken away were U.S. citizens. Nationwide, immigration officials have detained more than 170 American citizens, including 20 held for more than 24 hours without the ability to make a phone call, ProPublica reported.
+These actions are undermining the public trust that is necessary for effective enforcement of the nation’s immigration laws. The behavior of federal agents is provoking an angry backlash in many of the communities that Mr. Trump claims he is trying to help. If all of this is supposed to convey a sense of renewed law and order, it is not working.
+As is typical for Mr. Trump, he has identified a real problem — illegal immigration — but responded with a destructive solution. For decades, the United States tolerated a level of illegal immigration that fostered a sense of lawlessness at the border and frustrated many Americans, including many Latinos. The Biden administration’s porous policies worsened the situation, making possible the largest immigration surge in American history, with most of the arrivals lacking legal permission to enter the country. Mr. Trump campaigned on a promise to reverse those policies, and he has an electoral mandate to do so. At the border, he has succeeded at reducing illegal entries to the lowest levels in decades.
+Yet he does not have a mandate to treat people cruelly or to break the law himself. Polls show that most Americans disapprove of his handling of the issue. The country does not need to choose between the chaos of the Biden approach and the chaos of the Trump approach. The best solution remains a comprehensive law that secures the border, deters future illegal entries, expands legal immigration and provides a pathway to citizenship for unauthorized migrants who have made their lives in the United States and are otherwise law-abiding members of society. Short of that — and Congress shows no signs of passing such a law — Mr. Trump can address illegal immigration in ways that are both more humane and effective. This country needs to enforce its laws without terrorizing innocent Americans and abandoning its values.
+Of the many problems with Trump immigration policies, two themes stand out: the brutality toward immigrants who are here illegally and the unfairness toward citizens and legal immigrants.
+People who entered this country illegally often did so at great risk to themselves, seeking a better life in the United States. They violated the law, yes, but the response should be proportional to their crimes. It should be both firm and humane. Instead, the Trump administration has reveled in harshness. Masked, plain-clothed Immigration and Customs Enforcement agents have tackled and body slammed people on the streets. Officials have launched raids into homes, destroying people’s property.
+In one video, a federal agent said to a group of Latinos, including a U.S. citizen: “You got no rights here. You’re an amigo, brother.” After that encounter, one agent told another, referring to the immigrants, “We’re going to end up shooting some of them.” In another video, an agent yelled “adios” to the concerned wife of a detained migrant before he shoved her into a wall and she collapsed. Other disturbing videos have filled social media.
+The tactics violate both the law and human decency. On the legal side, recent court decisions have emphasized that people accused of being here without permission have a constitutional right to some due process. That right is to all of our benefit: If the federal government could simply say that someone is in the country illegally without having to prove the claim, it could deport anyone with impunity. On the human side, a vast majority of these migrants have done nothing worse than come to the country illegally, in search of a better life. Federal agents should respond appropriately, not with the expectation that violence is necessary.
+Editors’ Picks
+‘It: Welcome to Derry’ Season 1 Premiere Recap: Nuclear Family
+Zadie Smith Considers Art in the Age of Relentless Progress
+Who Is Cameron Crowe Kidding With the Title of His Memoir?
+The second problem with the Trump approach is that its breadth inevitably sweeps up U.S. citizens and other legal residents. Federal officials are relying on racial profiling in a country where 20 percent of the population is Latino, most of whom are legal residents or citizens. The administration is able to do so because of Congress’s acquiescence on the topic and a wrongheaded ruling that the Supreme Court issued last month, upholding the use of racial profiling in the raids.
+The use of racial discrimination in law enforcement should be an affront to all Americans. Videos show that many federal agents believe that the burden of proof is on Latinos to show they are here legally, not on the government officials who are accusing them of a crime. During a raid in California, officials yanked George Retes, a U.S. citizen who served in Iraq, from his car and held him for three days. Mr. Retes said he had a government ID in his vehicle, but officials did not let him show it to them. Similar treatment befell Javier Ramirez in California, Julio Noriega in Illinois and an unnamed military veteran in New Jersey, among others.
+Americans have responded to these problems with protests. As if to prove the protesters’ point, federal agents have reacted with more abuses of power, using tear gas and pepper balls on peaceful demonstrators. Even after a federal judge demanded an end to these practices, they have continued.
+Federal agents’ masks exacerbate the problems. Agents with masks know they are more likely to get away with violence and abuses of power because they are anonymous. To the community, masks signal that the government cares more about protecting its agents’ identities than democratic accountability. They create a sense that the government is sending faceless storm troopers to terrorize families.
+Despite its aggressiveness, the crackdown has not even been effective at dealing with the millions of people who are in this country without legal permission. The administration is missing its own deportation benchmarks. It is on pace to deport fewer people than the Obama administration did in some years. The Obama administration’s approach made sense. It focused on people who arrived recently and on those who had committed crimes since arriving in this country — and it typically respected people’s rights to due process. It did not resort to masked agents and violent raids.
+What separates democracy from authoritarianism, the rule of law from lawlessness and a decent society from an indecent one is not just the goal but the process. The government can, and should, reduce illegal immigration, but it should do so in a way that upholds American ideals.</t>
+  </si>
+  <si>
+    <t>https://www.nytimes.com/video/opinion/100000010479597/the-supreme-court-owes-the-country-an-explanation-for-its-big-decisions.html</t>
+  </si>
+  <si>
+    <t>You’ve seen the ICE raids, masked agents grabbing people who they think might be undocumented, sometimes only on the basis of skin color. “I’m from Brooklyn!” Or because they were speaking Spanish. How can this possibly be legal in the United States of America? “More fear.” “Terrorizing communities.” “170 U.S. citizens were detained by Homeland Security.” Well, it became legal just six weeks ago, when the Supreme Court gave ICE the green light to use racial profiling to decide who they suspect is undocumented. What made the Supreme Court’s decision so concerning wasn’t just how the court ruled, but also how little explanation the public received. The court held no oral arguments. They didn’t reveal the vote count, and the majority’s explanation amounted to little more than because we said so. Like so many recent decisions from the Supreme Court, this decision was delivered through a shortcut called the emergency docket. It’s meant for emergencies, but the Trump administration has been using it over and over again to expand the powers of the presidency, and the Supreme Court is playing along. This is the opinion of the New York Times editorial board. When the Supreme Court releases a normal merits docket decision —— “Here it is. Let’s take a look at it.” They outline their reasoning in dozens of pages. Pages that my colleague Emily Bazelon spends a lot of time reading. There’s one opinion for the majority: a rendition of the facts. Why the court has jurisdiction, what the lower courts have ruled previously, the legal analysis, which statutes or provisions of the Constitution they think are relevant, why they apply, the dissenting opinion, the kind of challenge to the majority opinion. There’s a kind of back and forth trying to expose each other’s weaknesses. So what’s the point of all these words? Fundamentally, showing their work so we understand what they’re doing. That is the basis of the judiciary’s authority. It’s how we know that what they’re doing is legitimate. Now, all of this writing and debating takes time, but on rare occasions, the court needs to move quickly, which is why the Supreme Court invented the emergency docket. Those faced with a lower court ruling that could cause great harm have the opportunity to ask the Supreme Court for emergency relief. For most of the country’s history, it was very rare for a presidential administration to ask for emergency relief. Bush asked for it five times and Obama only three times. Before that, the emergency docket used to be used almost entirely for one type of case. If you have your execution scheduled sometimes at midnight on the day that you’re going to the Supreme Court, it’s truly life or death. You cannot afford to wait. But today, the Trump administration has been using the emergency docket at an unprecedented rate, applying for emergency relief nearly 30 times since January. When one of his executive orders is deemed unlawful by a lower court, the Trump administration asks the Supreme Court for emergency relief, and time and time again, the conservative supermajority has taken the case and sided with the Trump administration, often leaving the American public with little explanation. “The court said the Trump administration can continue indiscriminate immigration stops targeting Latinos and Spanish speakers.” “To allow members of the Department of Government Efficiency to access personal information on millions of Americans ——” “Can cancel temporary protections for nearly 350,000 Venezuelan migrants.” “It’s not just that they’re overturning some of these decisions; it’s that they’re not really explaining why.” Most of these emergency docket decisions look like this. A single paragraph with little or no explanation. One way to think about this is all the examples in our lives when it helps to have explanations for what’s happening. So you get a paper back that you wrote in school and it just has a grade on it, but you don’t know what the teacher’s reasons were for giving you that grade. Especially if you didn’t get an A, you’re wondering: What did I do wrong? How could I improve on this? What if you get arrested and the police don’t tell you why? You’re not sure what you did wrong. To understand how these decisions are changing the powers of the presidency, just look at what happened with the Department of Education. All throughout the campaign, Trump made his intentions clear. “I’m going to close the Department of Education and move education back to the states.” But as president, he doesn’t actually have the authority to do that. Only Congress does. But that didn’t stop Trump. “President Trump just now signing that executive order to gut the Department of Education ——” Whole units of the Department of Ed get dismantled. There’s just nobody there to do the work anymore. So states and school districts sued, claiming it was unconstitutional. The lower courts agreed with the people who were challenging the executive order. But when the case reached the Supreme Court, the Supreme Court, on its emergency docket in this very brief, unsigned order, allowed the president to take these steps. And so we’re left wondering why. It’s just a big question mark. This opinion creates a precedent that the president can effectively dismantle a federal agency through mass firings With free speech, free press, open courtrooms and the right to due process, America has long been a land where we show our work, rather than hide it in the shadows. That the nation’s top court has suddenly excused itself from this tradition of transparency is alarming. Overuse of the emergency docket, it’s concentrating power in the hands of the president by ruling on his behalf, and by making itself the place deciding these questions, it’s also concentrating power in its own hands.</t>
+  </si>
+  <si>
+    <t>https://www.nytimes.com/2025/10/20/opinion/moderation-strategy-democrat-republican-center.html</t>
+  </si>
+  <si>
+    <t>American politics today can seem to be dominated by extremes. President Trump is carrying out far-right policies, while some of the country’s highest-profile Democrats identify as democratic socialists. Moderation sometimes feels outdated.
+It is not. Candidates closer to the political center, from both parties, continue to fare better in most elections than those farther to the right or left. This pattern may be the strongest one in electoral politics today, but it is one that many partisans try to obscure and many voters do not fully grasp.
+The evidence is vast. Republicans have frittered away winnable races in Alabama, New Hampshire and elsewhere over the past decade by nominating extremist candidates, while Senator Susan Collins of Maine, a moderate Republican, is the only sitting senator who represents a state that reliably votes the other way in presidential elections. On the Democratic side, there are no progressives in the mold of Alexandria Ocasio-Cortez or Bernie Sanders who represent a swing district or state. Instead, the Democrats who win tough races work hard to signal to voters that they are less progressive than their party.
+One way to see the pattern is to examine the 17 Democrats — 13 in the House, four in the Senate — who last year won in places that Mr. Trump also won. Moderation dominated their campaign messages. Ruben Gallego of Arizona mocked the term “Latinx” and was hawkish on immigration. Representative Vicente Gonzalez of Texas and Senator Jacky Rosen of Nevada criticized other Democrats’ tolerance of illegal immigration. Elissa Slotkin of Michigan and Representative Pat Ryan of New York emphasized public safety and their national security backgrounds. Senator Tammy Baldwin of Wisconsin bragged about taking on federal bureaucrats who had imposed needless regulation. Representative Jared Golden of Maine spoke of “opening up oil and gas production to lower fuel costs.” No progressive won a race as difficult as any of these.
+Left-wing Democrats and right-wing Republicans have spent years trying to tell a different story. They claim that reaching out to swing voters is overrated and that the better strategy involves turning out the base by running pure, ideological campaigns. They are wrong, but their argument does contain an element of truth: As the country has become more polarized and many voters cannot fathom crossing over to the other party, persuasion has become harder. It is not impossible, though — and it remains far more effective than pursuing the fantasy that America has a latent left-wing or right-wing majority waiting to be inspired to turn out.
+Even Mr. Trump highlights the pattern. Extreme as he is in many ways, he moved the Republican Party toward the center on several key issues. He won the party’s nomination and the general election in 2016 partly by rejecting unpopular conservative positions on Social Security, Medicare and global trade. Last year he broke with prominent Republicans and said he would veto a national abortion ban. He also focused his 2024 campaign on areas in which the Democratic Party had moved left over the previous decade and was out of step with public opinion, such as immigration, transgender issues and parts of education policy. Voters noticed. Polls in 2024 showed that most voters considered their policy views to be closer to Mr. Trump’s than to Kamala Harris’s.
+Mr. Trump’s victory over Ms. Harris was telling in another way. The moderation that has worked best in recent years is not a sober, 20th-century centrism that promises to protect the status quo. It is more combative and populist. It tends to be left of center on economics and right of center on social issues (with abortion being an exception). “Angry centrism is a very potent way to run,” said Lakshya Jain, a founder of Split Ticket, a political data firm. Rather than locating itself midway between the two parties, this new centrism promises sweeping change while criticizing the two parties as out of touch.
+As Representative Marcy Kaptur, Democrat of Ohio, said in a campaign ad last year, “America has gotten off course.” She cited “the far left ignoring millions illegally crossing the border and trying to defund the police” and “the far right taking away women’s rights and protecting greedy corporations at every turn.” Although Mr. Trump won her district by seven percentage points, voters re-elected her.
+The success of candidates like her demonstrates that America still has a political center. Polls show that most voters prefer capitalism to socialism and worry that the government is too big — and also think that corporations and the wealthy have too much power. Most voters oppose both the cruel immigration enforcement of the Trump administration and the lax Biden policies that led to a record immigration surge. Most favor robust policing to combat crime and recoil at police brutality. Most favor widespread abortion access and some restrictions late in pregnancy. Most oppose race-based affirmative action and support class-based affirmative action. Most support job protections for trans people and believe that trans girls should not play girls’ sports. Most want strong public schools and the flexibility to choose which school their children attend.
+Apart from individual issues, many voters understand the importance of political independence for its own sake. A diverse, pluralistic nation depends on mutual understanding and regular compromise. Our political system works best when it includes politicians who are not beholden to either side’s orthodoxy and instead build coalitions to tackle major challenges. It is no coincidence that as the number of heterodox, compromise-oriented Democrats and Republicans has declined in Washington, Congress has become less functional.
+These lessons are especially urgent for Democrats. Despite Mr. Trump’s rhetorical nods to the center, he is governing as a radical who rejects longstanding governing constraints and uses the power of the presidency to enrich his family, protect his allies and punish people he dislikes. He threatens American democracy, and congressional Republicans have been complicit. The Democratic Party, as a result, has become the only party of the country’s two major ones that respects basic republican traditions like the sanctity of elections and the constitutional system of checks and balances.
+Yet many Americans see the Democratic Party as too liberal, too judgmental and too focused on cultural issues to be credible, and voters are moving away from it. “Of the 30 states that track voter registration by political party, Democrats lost ground to Republicans in every single one between the 2020 and 2024 elections — and often by a lot,” The Times reported this summer. Perhaps most worrisome for Democrats, younger voters, nonwhite Americans and immigrants, all growing parts of the electorate, have shifted from the party.
+Many progressives have tried to wish away these warning signs and insist that they can win by quietly retaining all their unpopular positions and emphasizing economic issues. But they cannot point to a single member of Congress or governor from swing districts or states who has pursued this strategy and won. Their favorite examples are all from deep blue parts of the country. The failure of the motivate-the-base approach is hiding in plain sight.
+Georgia and Wisconsin have offered recent case studies. In Georgia, Raphael Warnock and Stacey Abrams, both Democrats, ran for statewide offices in 2022, making what NBC News called “two markedly different pitches to voters.” She ran a “bold progressive” campaign meant to “turbocharge progressive turnout,” while he put “a greater emphasis on courting the center” by emphasizing his independence and bipartisanship. He won his Senate race. She lost her race for governor, as she did four years earlier. Likewise, in Wisconsin, Mandela Barnes, a progressive Democrat with a history of supporting cuts to immigration enforcement and police funding, lost his 2022 Senate race, while Ms. Baldwin and Gov. Tony Evers have won by running to the middle.</t>
+  </si>
+  <si>
+    <t>https://www.nytimes.com/2025/10/17/opinion/russia-ukraine-war-nato-putin.html</t>
+  </si>
+  <si>
+    <t>Russia has launched a new and dangerous campaign of provocation against NATO. Over the past six weeks, it has sent drones over Poland and Romania and flown fighter jets into Estonia. Russia was also very likely behind drone flights that disrupted activity at airports in Denmark, Belgium and Germany. President Vladimir Putin has unconvincingly denied responsibility for all these acts and in fact seems happy for the world to believe Russia is behind them.
+His goals are to scare, exhaust and divide Europeans, causing them to question their support for Ukraine and undermine its efforts to repel Russia’s invasion. Ultimately, he also wants to make the United States look weak and fragment the NATO alliance. Responding wisely to him is vital for Washington and Europe. It is not easy. Striking back hard risks escalating conflict, while doing nothing conveys a weakness that invites future aggression.
+NATO allies are aware that Russia is testing them and so far have done a good job of responding. They have denounced the incursions, forthrightly blamed Russia for them and met this month in Copenhagen in a show of unity. “We are not at war,” Chancellor Friedrich Merz of Germany said recently, “but we are no longer at peace either.”
+There is more to do. European leaders should make clear that Russian aggression against NATO countries risks a forceful response, including the shooting down of drones — as the West has already done — and potentially of Russian fighter planes that enter NATO airspace.
+The United States and its NATO allies should also use the new Russian aggression as a reason to increase their support for Ukraine, sending the message that Mr. Putin’s attempt to weaken Western resolve has backfired. The visit this Friday of President Volodymyr Zelensky of Ukraine to the White House is an opportunity for President Trump to commit to new military and economic aid for Kyiv.
+All these responses bring risks, including the dangers of escalation. By now, though, the world should know that there are no safe options with Mr. Putin. Ignoring or downplaying his aggressions encourages more of them. If he comes to believe that he can menace Poland, Estonia and other NATO members without consequence, he will become bolder about doing so.
+“We must not only react, we must deter,” said Ursula von der Leyen, the European Commission president. “Because if we hesitate to act, the gray zone will only expand.” She is right. Sometimes, the best way to prevent military escalation is to draw a firm line.
+The latest Russian provocations began on Sept. 9 with more than a dozen drones that crossed into Poland after having flown over Belarus and Ukraine. Five days later, a drone crossed into Romania, near two Romanian fighters on patrol. Five days after that, three Russian MiG jets flew into Estonia.
+Then came a mysterious intrusion of civilian drones around commercial airports. The week after the Estonian incident, several drones flew near two airports in Denmark in what the country’s defense minister called a “hybrid attack,” and officials briefly closed the airports to avoid the risk of a crash. Drones later disrupted air travel in Belgium and Germany.
+NATO responded well to these provocations. The MiGs over Estonia created the thorniest problem because they raised the prospect of a military confrontation between human pilots. But Swedish and Finnish pilots engaged with the MiGs, and the Russian pilots stood down, leaving Estonia escorted by the NATO planes. The response to the drones was even more aggressive. A combination of Polish, Dutch, Italian and German pilots intercepted the drones flying over Poland, shooting down several of them. In Romania, pilots tracked the Russian drone, and it left NATO airspace on its own.
+One downside to destroying drones is that it can be expensive. Some of the missiles that NATO used cost $1 million, many times more than a drone. To address this problem, NATO should expand the production of armed drones, develop more effective electronic warfare defenses against them and fund research into other countermeasures. Russian aggression should serve as a reminder that warfare is changing and that defense industries must change with it.
+As for future intrusions by piloted Russian jets, some Eastern European countries are arguing for loosening the rules for how and when NATO pilots can confront Russian jets that enter alliance airspace. A mix of caution and firmness is the best course. Nobody wants direct conflict between NATO and Russia, but history shows that the use of force can lead Mr. Putin to pull back. In the mid-2010s, Russian jets sometimes flew over Turkey, and Turkey, a NATO member, told Russia to stop. Only after Turkey downed a jet did Russia retreat.
+It is also important to respond in the theater that Mr. Putin cares about most: Ukraine. The incursions appear to have been partly a reaction to recent American equivocation. They came less than a month after an Alaska summit during which Mr. Putin succeeded in getting Mr. Trump to step back from his efforts to pressure Russia into accepting a cease-fire in Ukraine. Europe was rightly disappointed.
+Still, if Mr. Putin thought that Alaska provided an opening to further divide the allies, he miscalculated. In response to the incursions, and perhaps thanks to the lack of diplomatic progress, Mr. Trump has expressed growing frustration. He said last month that Mr. Putin “has really let me down.” Mr. Trump also said that NATO planes should shoot down Russian aircraft that enter allied airspace and raised the possibility of new forms of support for Ukraine.
+Already, he has authorized more intelligence sharing with Kyiv to heighten the effectiveness of its attacks, including those on Russian oil and gas facilities. Another option involves allowing Ukraine to get Tomahawk missiles. The missiles have a 1,000-mile range, and Ukraine could use them to strike deeper inside Russia.
+Mr. Trump’s history of impulsiveness and his long record of coziness with Mr. Putin offer reasons to remain skeptical that this new posture will be a lasting one. On Thursday, the two leaders spent more than two hours on the phone together, and Mr. Trump described the conversation as “very productive.” They plan to follow up by meeting in Budapest soon.
+That meeting will be an opportunity to draw a firm line. Russia’s recent aggression toward NATO shows that Russia’s war in Ukraine is about much more than Ukraine. It is about Mr. Putin’s revanchist ambitions in Europe. The only way to contain him is with resolute strength.</t>
+  </si>
+  <si>
+    <t>https://www.nytimes.com/2025/10/10/opinion/letitia-james-indictment-trump.html</t>
+  </si>
+  <si>
+    <t>President Trump is once again weaponizing the legal system to fulfill his personal vendettas. Last year, before he could point to a single crime that he claimed she had committed, Mr. Trump called for the prosecution of New York’s attorney general, Letitia James, who was suing him for fraudulent business dealing. On Thursday the Justice Department secured an indictment against Ms. James, alleging bank fraud.
+The story behind the indictment says it all. A federal prosecutor decided recently that there was not enough evidence to bring charges against Ms. James. In a normal administration, that would have been the end of the case. But Mr. Trump did not take no for an answer. He forced that prosecutor’s resignation and in a social media post last month demanded that Attorney General Pam Bondi appoint a new prosecutor: Lindsey Halligan, a Trump ally and insurance lawyer who had never prosecuted a case.
+He also demanded that Ms. Halligan pursue charges against both Ms. James and James Comey, the former director of the F.B.I. “They impeached me twice, and indicted me (5 times!), OVER NOTHING,” Mr. Trump wrote on Truth Social. “JUSTICE MUST BE SERVED, NOW!!!” At Ms. Halligan’s request, a grand jury indicted Mr. Comey on Sept. 25 and then Ms. James.
+The charges relate to mortgage paperwork that Ms. James filed when she bought a house in Virginia in 2020. Previous prosecutors did not find sufficient evidence that Ms. James was knowingly dishonest, and legal experts say the charges are flimsy at best. Even if the Justice Department ultimately loses in court, the legal fight will demand Ms. James’s time and money. It signals to politicians and the public that opposing the president has a cost, including the explicit threat of imprisonment.
+Mr. Trump and his supporters claim that Democrats started this era of “lawfare” with their investigations into him. Yet those investigations were vastly different. Special counsels, chosen to operate more independently than typical prosecutors, carried out the federal inquiries into Mr. Trump. One special counsel during the Biden administration even investigated Joe Biden himself for his handling of classified documents. And the investigations into Mr. Trump came in response to his alarming actions, not dubious claims of mortgage problems but efforts to overturn the outcome of a presidential election. The investigations followed a potential crime, not a personal vendetta.
+America is now in a dangerous period, in which the president can order investigations and indictments against his enemies. Mr. Trump is criminalizing Americans’ ability to challenge their leaders.
+In the popular imagination, the state’s infringement on individual liberty is usually the work of spies or the military. But few branches of government have the power to take away our freedoms that the Justice Department does. It can ask courts to put you in prison, mark your life with a criminal record and, even if you are found not guilty, tie you up in yearslong legal battles that drain your finances and destroy your personal standing. “The prosecutor has more control over life, liberty and reputation than any other person in America,” former Supreme Court Justice Robert Jackson said when he served as attorney general.
+Cognizant of these concerns, presidents since Watergate have mostly tried to insulate the Justice Department from politics. The system has not been perfect, but it has mostly worked. Americans have generally trusted the federal government to avoid sham prosecutions.
+Mr. Trump has eroded this system from within. His replacement of a career prosecutor with a crony is only one example. He has staffed the Justice Department and the F.B.I. with loyalists. His administration has pushed out lawyers who investigated misconduct and corruption. He has tried to punish law firms that represent his political opponents. He has repeatedly warned officials, sometimes in public social media posts, that they should not go against him. He has sent a message that federal law enforcement’s main concern should be not the country’s laws or the Constitution but his personal interests.
+Editors’ Picks
+Let Us Help You Find Your Next Children’s Book
+How to Deal With 30 to 50 Feral Hogs
+What Inspires the Best Costumes at Comic Con? A Little Childhood Trauma.
+Just as telling as the cases Mr. Trump’s Justice Department has initiated are those it has dropped. This year the department closed an investigation into Tom Homan, the president’s so-called border czar, even though he was recorded accepting a bag of $50,000 in cash by undercover F.B.I. agents.
+Many legal experts have spoken out. “These political prosecutions need to stop,” wrote Richard Painter, who was a White House ethics lawyer under George W. Bush, after Ms. James was indicted. He called for an impeachment inquiry into Ms. Bondi. Most Republicans, however, have remained quiet, fearful of the president.
+Mr. Comey and Ms. James’s indictments may be just the beginning. Mr. Trump has also demanded the prosecution of one of his most prominent Democratic opponents, Senator Adam Schiff of California. He posted on social media this week that Gov. JB Pritzker of Illinois and Mayor Brandon Johnson of Chicago should go to jail for opposing his mass deportation efforts. His Justice Department has proved all too willing to turn such social media posts, no matter how baseless, into indictments.
+The damage is not just to Mr. Comey, Ms. James and anyone else who is prosecuted. It is also to the foundations of American democracy and law.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -116,7 +232,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -129,8 +245,20 @@
         <bgColor rgb="FFBDBDBD"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF3F3F3"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -138,21 +266,97 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -396,7 +600,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
@@ -404,57 +608,81 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-    </row>
-    <row r="5" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
+    <row r="4" spans="1:2" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="6" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-    </row>
-    <row r="7" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-    </row>
-    <row r="8" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-    </row>
-    <row r="9" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-    </row>
-    <row r="10" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
-    </row>
-    <row r="11" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-    </row>
-    <row r="12" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
-    </row>
-    <row r="13" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
+      <c r="A6" s="6"/>
+      <c r="B6" s="6"/>
+    </row>
+    <row r="7" spans="1:2" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="7"/>
+      <c r="B7" s="7"/>
+    </row>
+    <row r="8" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="9"/>
+      <c r="B9" s="11"/>
+    </row>
+    <row r="10" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="11"/>
+      <c r="B11" s="11"/>
+    </row>
+    <row r="12" spans="1:2" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="14" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
+      <c r="A14" s="6"/>
+      <c r="B14" s="6"/>
     </row>
     <row r="15" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-    </row>
-    <row r="16" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
+      <c r="A15" s="6"/>
+      <c r="B15" s="6"/>
+    </row>
+    <row r="16" spans="1:2" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="7"/>
+      <c r="B16" s="7"/>
     </row>
     <row r="17" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
@@ -4398,11 +4626,22 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:B1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <mergeCells count="8">
+    <mergeCell ref="A13:A16"/>
+    <mergeCell ref="B13:B16"/>
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="B10:B11"/>
+  </mergeCells>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1" xr:uid="{89488486-3D04-43A0-BC57-26D0D3B1C37F}"/>
     <hyperlink ref="A3" r:id="rId2" xr:uid="{3CBB89FD-6531-4F6D-A1C8-96F35FBF0B7B}"/>
+    <hyperlink ref="A8" r:id="rId3" xr:uid="{14B38C14-62A7-4A9F-AC90-487844A58591}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
-  <pageSetup orientation="landscape"/>
+  <pageSetup orientation="landscape" r:id="rId4"/>
 </worksheet>
 </file>
</xml_diff>